<commit_message>
Add a machine-by-package sheet to the sample data
A cross-reference of which machine can run which package, marking the
kit each one currently holds, with five formula rows underneath that
compare each package's workload against the sites currently configured
for it.

The last row is the point: workload divided by currently-mounted sites
says how long each package would take if the fleet never changed a kit.
For this dataset QFN32 needs 7.0 hours against a 4.0-hour fleet average,
which is why minimising changeovers strands it.

The sheet is a view of the 機台 sheet; the loader still reads that one.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TrwTqMZ3kHRLL23LGZ4TZk
</commit_message>
<xml_diff>
--- a/docs/模擬WIP_200批.xlsx
+++ b/docs/模擬WIP_200批.xlsx
@@ -10,6 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="說明" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="貨批" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="機台" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="能力矩陣" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -18,10 +19,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="#,##0.0"/>
+    <numFmt numFmtId="165" formatCode="0.0"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -69,8 +71,14 @@
       <color rgb="00C2410C"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="001C7293"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -90,6 +98,16 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="001E2761"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF1CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFE8D9"/>
       </patternFill>
     </fill>
   </fills>
@@ -119,7 +137,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -144,6 +162,22 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -10303,4 +10337,1132 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J38"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="7" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="11" t="inlineStr">
+        <is>
+          <t>機台</t>
+        </is>
+      </c>
+      <c r="B1" s="11" t="inlineStr">
+        <is>
+          <t>sites</t>
+        </is>
+      </c>
+      <c r="C1" s="11" t="inlineStr">
+        <is>
+          <t>QFN48</t>
+        </is>
+      </c>
+      <c r="D1" s="11" t="inlineStr">
+        <is>
+          <t>QFN32</t>
+        </is>
+      </c>
+      <c r="E1" s="11" t="inlineStr">
+        <is>
+          <t>SOP16</t>
+        </is>
+      </c>
+      <c r="F1" s="11" t="inlineStr">
+        <is>
+          <t>TSSOP28</t>
+        </is>
+      </c>
+      <c r="G1" s="11" t="inlineStr">
+        <is>
+          <t>BGA144</t>
+        </is>
+      </c>
+      <c r="H1" s="11" t="inlineStr">
+        <is>
+          <t>目前裝著的 Kit</t>
+        </is>
+      </c>
+      <c r="I1" s="11" t="inlineStr">
+        <is>
+          <t>目前程式</t>
+        </is>
+      </c>
+      <c r="J1" s="11" t="inlineStr">
+        <is>
+          <t>幾小時後可用</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="9" t="inlineStr">
+        <is>
+          <t>T01</t>
+        </is>
+      </c>
+      <c r="B2" s="12" t="n">
+        <v>8</v>
+      </c>
+      <c r="C2" s="13" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="D2" s="14" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="E2" s="14" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="F2" s="14" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="G2" s="14" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="H2" s="9" t="inlineStr">
+        <is>
+          <t>QFN48</t>
+        </is>
+      </c>
+      <c r="I2" s="9" t="inlineStr">
+        <is>
+          <t>MCU01_V3</t>
+        </is>
+      </c>
+      <c r="J2" s="12" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="9" t="inlineStr">
+        <is>
+          <t>T02</t>
+        </is>
+      </c>
+      <c r="B3" s="12" t="n">
+        <v>8</v>
+      </c>
+      <c r="C3" s="14" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="D3" s="13" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="E3" s="14" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="F3" s="14" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="G3" s="14" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="H3" s="9" t="inlineStr">
+        <is>
+          <t>QFN32</t>
+        </is>
+      </c>
+      <c r="I3" s="9" t="inlineStr">
+        <is>
+          <t>PMIC09_V1</t>
+        </is>
+      </c>
+      <c r="J3" s="12" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="9" t="inlineStr">
+        <is>
+          <t>T03</t>
+        </is>
+      </c>
+      <c r="B4" s="12" t="n">
+        <v>8</v>
+      </c>
+      <c r="C4" s="14" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="D4" s="14" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="E4" s="13" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="F4" s="14" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="G4" s="14" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="H4" s="9" t="inlineStr">
+        <is>
+          <t>SOP16</t>
+        </is>
+      </c>
+      <c r="I4" s="9" t="inlineStr">
+        <is>
+          <t>LED03_V1</t>
+        </is>
+      </c>
+      <c r="J4" s="12" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="9" t="inlineStr">
+        <is>
+          <t>T04</t>
+        </is>
+      </c>
+      <c r="B5" s="12" t="n">
+        <v>8</v>
+      </c>
+      <c r="C5" s="14" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="D5" s="14" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="E5" s="14" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="F5" s="13" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="G5" s="14" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="H5" s="9" t="inlineStr">
+        <is>
+          <t>TSSOP28</t>
+        </is>
+      </c>
+      <c r="I5" s="9" t="inlineStr">
+        <is>
+          <t>SENS11_V4</t>
+        </is>
+      </c>
+      <c r="J5" s="12" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>T05</t>
+        </is>
+      </c>
+      <c r="B6" s="12" t="n">
+        <v>8</v>
+      </c>
+      <c r="C6" s="14" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="D6" s="14" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="E6" s="14" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="F6" s="14" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="G6" s="13" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="H6" s="9" t="inlineStr">
+        <is>
+          <t>BGA144</t>
+        </is>
+      </c>
+      <c r="I6" s="9" t="inlineStr">
+        <is>
+          <t>SOC22_V2</t>
+        </is>
+      </c>
+      <c r="J6" s="12" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="9" t="inlineStr">
+        <is>
+          <t>T06</t>
+        </is>
+      </c>
+      <c r="B7" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="C7" s="13" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="D7" s="15" t="inlineStr"/>
+      <c r="E7" s="15" t="inlineStr"/>
+      <c r="F7" s="15" t="inlineStr"/>
+      <c r="G7" s="15" t="inlineStr"/>
+      <c r="H7" s="9" t="inlineStr">
+        <is>
+          <t>QFN48</t>
+        </is>
+      </c>
+      <c r="I7" s="9" t="inlineStr">
+        <is>
+          <t>MCU01_V3</t>
+        </is>
+      </c>
+      <c r="J7" s="12" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="9" t="inlineStr">
+        <is>
+          <t>T07</t>
+        </is>
+      </c>
+      <c r="B8" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="C8" s="13" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="D8" s="15" t="inlineStr"/>
+      <c r="E8" s="15" t="inlineStr"/>
+      <c r="F8" s="15" t="inlineStr"/>
+      <c r="G8" s="15" t="inlineStr"/>
+      <c r="H8" s="9" t="inlineStr">
+        <is>
+          <t>QFN48</t>
+        </is>
+      </c>
+      <c r="I8" s="9" t="inlineStr">
+        <is>
+          <t>MCU01_V3</t>
+        </is>
+      </c>
+      <c r="J8" s="12" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="9" t="inlineStr">
+        <is>
+          <t>T08</t>
+        </is>
+      </c>
+      <c r="B9" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="C9" s="13" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="D9" s="15" t="inlineStr"/>
+      <c r="E9" s="15" t="inlineStr"/>
+      <c r="F9" s="15" t="inlineStr"/>
+      <c r="G9" s="15" t="inlineStr"/>
+      <c r="H9" s="9" t="inlineStr">
+        <is>
+          <t>QFN48</t>
+        </is>
+      </c>
+      <c r="I9" s="9" t="inlineStr">
+        <is>
+          <t>MCU01_V3</t>
+        </is>
+      </c>
+      <c r="J9" s="12" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="9" t="inlineStr">
+        <is>
+          <t>T09</t>
+        </is>
+      </c>
+      <c r="B10" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="C10" s="13" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="D10" s="15" t="inlineStr"/>
+      <c r="E10" s="15" t="inlineStr"/>
+      <c r="F10" s="15" t="inlineStr"/>
+      <c r="G10" s="15" t="inlineStr"/>
+      <c r="H10" s="9" t="inlineStr">
+        <is>
+          <t>QFN48</t>
+        </is>
+      </c>
+      <c r="I10" s="9" t="inlineStr">
+        <is>
+          <t>MCU02_V1</t>
+        </is>
+      </c>
+      <c r="J10" s="12" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="9" t="inlineStr">
+        <is>
+          <t>T10</t>
+        </is>
+      </c>
+      <c r="B11" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="C11" s="13" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="D11" s="15" t="inlineStr"/>
+      <c r="E11" s="15" t="inlineStr"/>
+      <c r="F11" s="15" t="inlineStr"/>
+      <c r="G11" s="15" t="inlineStr"/>
+      <c r="H11" s="9" t="inlineStr">
+        <is>
+          <t>QFN48</t>
+        </is>
+      </c>
+      <c r="I11" s="9" t="inlineStr">
+        <is>
+          <t>MCU01_V3</t>
+        </is>
+      </c>
+      <c r="J11" s="12" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="9" t="inlineStr">
+        <is>
+          <t>T11</t>
+        </is>
+      </c>
+      <c r="B12" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="C12" s="13" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="D12" s="15" t="inlineStr"/>
+      <c r="E12" s="15" t="inlineStr"/>
+      <c r="F12" s="15" t="inlineStr"/>
+      <c r="G12" s="15" t="inlineStr"/>
+      <c r="H12" s="9" t="inlineStr">
+        <is>
+          <t>QFN48</t>
+        </is>
+      </c>
+      <c r="I12" s="9" t="inlineStr">
+        <is>
+          <t>MCU01_V3</t>
+        </is>
+      </c>
+      <c r="J12" s="12" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="9" t="inlineStr">
+        <is>
+          <t>T12</t>
+        </is>
+      </c>
+      <c r="B13" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="C13" s="13" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="D13" s="15" t="inlineStr"/>
+      <c r="E13" s="15" t="inlineStr"/>
+      <c r="F13" s="15" t="inlineStr"/>
+      <c r="G13" s="15" t="inlineStr"/>
+      <c r="H13" s="9" t="inlineStr">
+        <is>
+          <t>QFN48</t>
+        </is>
+      </c>
+      <c r="I13" s="9" t="inlineStr">
+        <is>
+          <t>MCU02_V1</t>
+        </is>
+      </c>
+      <c r="J13" s="12" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="9" t="inlineStr">
+        <is>
+          <t>T13</t>
+        </is>
+      </c>
+      <c r="B14" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="C14" s="13" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="D14" s="15" t="inlineStr"/>
+      <c r="E14" s="15" t="inlineStr"/>
+      <c r="F14" s="15" t="inlineStr"/>
+      <c r="G14" s="15" t="inlineStr"/>
+      <c r="H14" s="9" t="inlineStr">
+        <is>
+          <t>QFN48</t>
+        </is>
+      </c>
+      <c r="I14" s="9" t="inlineStr">
+        <is>
+          <t>MCU01_V5</t>
+        </is>
+      </c>
+      <c r="J14" s="12" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="9" t="inlineStr">
+        <is>
+          <t>T14</t>
+        </is>
+      </c>
+      <c r="B15" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="C15" s="15" t="inlineStr"/>
+      <c r="D15" s="13" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="E15" s="15" t="inlineStr"/>
+      <c r="F15" s="15" t="inlineStr"/>
+      <c r="G15" s="15" t="inlineStr"/>
+      <c r="H15" s="9" t="inlineStr">
+        <is>
+          <t>QFN32</t>
+        </is>
+      </c>
+      <c r="I15" s="9" t="inlineStr">
+        <is>
+          <t>PMIC09_V1</t>
+        </is>
+      </c>
+      <c r="J15" s="12" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="9" t="inlineStr">
+        <is>
+          <t>T15</t>
+        </is>
+      </c>
+      <c r="B16" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="C16" s="15" t="inlineStr"/>
+      <c r="D16" s="13" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="E16" s="15" t="inlineStr"/>
+      <c r="F16" s="15" t="inlineStr"/>
+      <c r="G16" s="15" t="inlineStr"/>
+      <c r="H16" s="9" t="inlineStr">
+        <is>
+          <t>QFN32</t>
+        </is>
+      </c>
+      <c r="I16" s="9" t="inlineStr">
+        <is>
+          <t>PMIC09_V1</t>
+        </is>
+      </c>
+      <c r="J16" s="12" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="9" t="inlineStr">
+        <is>
+          <t>T16</t>
+        </is>
+      </c>
+      <c r="B17" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="C17" s="15" t="inlineStr"/>
+      <c r="D17" s="13" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="E17" s="15" t="inlineStr"/>
+      <c r="F17" s="15" t="inlineStr"/>
+      <c r="G17" s="15" t="inlineStr"/>
+      <c r="H17" s="9" t="inlineStr">
+        <is>
+          <t>QFN32</t>
+        </is>
+      </c>
+      <c r="I17" s="9" t="inlineStr">
+        <is>
+          <t>PMIC09_V1</t>
+        </is>
+      </c>
+      <c r="J17" s="12" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="9" t="inlineStr">
+        <is>
+          <t>T17</t>
+        </is>
+      </c>
+      <c r="B18" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="C18" s="15" t="inlineStr"/>
+      <c r="D18" s="13" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="E18" s="15" t="inlineStr"/>
+      <c r="F18" s="15" t="inlineStr"/>
+      <c r="G18" s="15" t="inlineStr"/>
+      <c r="H18" s="9" t="inlineStr">
+        <is>
+          <t>QFN32</t>
+        </is>
+      </c>
+      <c r="I18" s="9" t="inlineStr">
+        <is>
+          <t>PMIC09_V1</t>
+        </is>
+      </c>
+      <c r="J18" s="12" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="9" t="inlineStr">
+        <is>
+          <t>T18</t>
+        </is>
+      </c>
+      <c r="B19" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="C19" s="15" t="inlineStr"/>
+      <c r="D19" s="13" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="E19" s="15" t="inlineStr"/>
+      <c r="F19" s="15" t="inlineStr"/>
+      <c r="G19" s="15" t="inlineStr"/>
+      <c r="H19" s="9" t="inlineStr">
+        <is>
+          <t>QFN32</t>
+        </is>
+      </c>
+      <c r="I19" s="9" t="inlineStr">
+        <is>
+          <t>PMIC07_V2</t>
+        </is>
+      </c>
+      <c r="J19" s="12" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="9" t="inlineStr">
+        <is>
+          <t>T19</t>
+        </is>
+      </c>
+      <c r="B20" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="C20" s="15" t="inlineStr"/>
+      <c r="D20" s="15" t="inlineStr"/>
+      <c r="E20" s="13" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="F20" s="15" t="inlineStr"/>
+      <c r="G20" s="15" t="inlineStr"/>
+      <c r="H20" s="9" t="inlineStr">
+        <is>
+          <t>SOP16</t>
+        </is>
+      </c>
+      <c r="I20" s="9" t="inlineStr">
+        <is>
+          <t>LED03_V1</t>
+        </is>
+      </c>
+      <c r="J20" s="12" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="9" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
+      <c r="B21" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="C21" s="15" t="inlineStr"/>
+      <c r="D21" s="15" t="inlineStr"/>
+      <c r="E21" s="13" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="F21" s="15" t="inlineStr"/>
+      <c r="G21" s="15" t="inlineStr"/>
+      <c r="H21" s="9" t="inlineStr">
+        <is>
+          <t>SOP16</t>
+        </is>
+      </c>
+      <c r="I21" s="9" t="inlineStr">
+        <is>
+          <t>LED03_V1</t>
+        </is>
+      </c>
+      <c r="J21" s="12" t="n">
+        <v>3.2</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="9" t="inlineStr">
+        <is>
+          <t>T21</t>
+        </is>
+      </c>
+      <c r="B22" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="C22" s="15" t="inlineStr"/>
+      <c r="D22" s="15" t="inlineStr"/>
+      <c r="E22" s="13" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="F22" s="15" t="inlineStr"/>
+      <c r="G22" s="15" t="inlineStr"/>
+      <c r="H22" s="9" t="inlineStr">
+        <is>
+          <t>SOP16</t>
+        </is>
+      </c>
+      <c r="I22" s="9" t="inlineStr">
+        <is>
+          <t>LED03_V1</t>
+        </is>
+      </c>
+      <c r="J22" s="12" t="n">
+        <v>1.4</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="9" t="inlineStr">
+        <is>
+          <t>T22</t>
+        </is>
+      </c>
+      <c r="B23" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="C23" s="15" t="inlineStr"/>
+      <c r="D23" s="15" t="inlineStr"/>
+      <c r="E23" s="13" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="F23" s="15" t="inlineStr"/>
+      <c r="G23" s="15" t="inlineStr"/>
+      <c r="H23" s="9" t="inlineStr">
+        <is>
+          <t>SOP16</t>
+        </is>
+      </c>
+      <c r="I23" s="9" t="inlineStr">
+        <is>
+          <t>LED03_V1</t>
+        </is>
+      </c>
+      <c r="J23" s="12" t="n">
+        <v>2.6</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="9" t="inlineStr">
+        <is>
+          <t>T23</t>
+        </is>
+      </c>
+      <c r="B24" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="C24" s="15" t="inlineStr"/>
+      <c r="D24" s="15" t="inlineStr"/>
+      <c r="E24" s="15" t="inlineStr"/>
+      <c r="F24" s="13" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="G24" s="15" t="inlineStr"/>
+      <c r="H24" s="9" t="inlineStr">
+        <is>
+          <t>TSSOP28</t>
+        </is>
+      </c>
+      <c r="I24" s="9" t="inlineStr">
+        <is>
+          <t>SENS11_V4</t>
+        </is>
+      </c>
+      <c r="J24" s="12" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="9" t="inlineStr">
+        <is>
+          <t>T24</t>
+        </is>
+      </c>
+      <c r="B25" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="C25" s="15" t="inlineStr"/>
+      <c r="D25" s="15" t="inlineStr"/>
+      <c r="E25" s="15" t="inlineStr"/>
+      <c r="F25" s="13" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="G25" s="15" t="inlineStr"/>
+      <c r="H25" s="9" t="inlineStr">
+        <is>
+          <t>TSSOP28</t>
+        </is>
+      </c>
+      <c r="I25" s="9" t="inlineStr">
+        <is>
+          <t>SENS11_V4</t>
+        </is>
+      </c>
+      <c r="J25" s="12" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="9" t="inlineStr">
+        <is>
+          <t>T25</t>
+        </is>
+      </c>
+      <c r="B26" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="C26" s="15" t="inlineStr"/>
+      <c r="D26" s="15" t="inlineStr"/>
+      <c r="E26" s="15" t="inlineStr"/>
+      <c r="F26" s="15" t="inlineStr"/>
+      <c r="G26" s="13" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
+      <c r="H26" s="9" t="inlineStr">
+        <is>
+          <t>BGA144</t>
+        </is>
+      </c>
+      <c r="I26" s="9" t="inlineStr">
+        <is>
+          <t>SOC22_V2</t>
+        </is>
+      </c>
+      <c r="J26" s="12" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>能測這種封裝的機台數</t>
+        </is>
+      </c>
+      <c r="C28" s="16">
+        <f>COUNTIF(C2:C26,"✔")</f>
+        <v/>
+      </c>
+      <c r="D28" s="16">
+        <f>COUNTIF(D2:D26,"✔")</f>
+        <v/>
+      </c>
+      <c r="E28" s="16">
+        <f>COUNTIF(E2:E26,"✔")</f>
+        <v/>
+      </c>
+      <c r="F28" s="16">
+        <f>COUNTIF(F2:F26,"✔")</f>
+        <v/>
+      </c>
+      <c r="G28" s="16">
+        <f>COUNTIF(G2:G26,"✔")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>能測這種封裝的 site 合計</t>
+        </is>
+      </c>
+      <c r="C29" s="16">
+        <f>SUMIF(C2:C26,"✔",$B$2:$B$26)</f>
+        <v/>
+      </c>
+      <c r="D29" s="16">
+        <f>SUMIF(D2:D26,"✔",$B$2:$B$26)</f>
+        <v/>
+      </c>
+      <c r="E29" s="16">
+        <f>SUMIF(E2:E26,"✔",$B$2:$B$26)</f>
+        <v/>
+      </c>
+      <c r="F29" s="16">
+        <f>SUMIF(F2:F26,"✔",$B$2:$B$26)</f>
+        <v/>
+      </c>
+      <c r="G29" s="16">
+        <f>SUMIF(G2:G26,"✔",$B$2:$B$26)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>目前正裝著這種 Kit 的 site</t>
+        </is>
+      </c>
+      <c r="C30" s="16">
+        <f>SUMIF($H$2:$H$26,C$1,$B$2:$B$26)</f>
+        <v/>
+      </c>
+      <c r="D30" s="16">
+        <f>SUMIF($H$2:$H$26,D$1,$B$2:$B$26)</f>
+        <v/>
+      </c>
+      <c r="E30" s="16">
+        <f>SUMIF($H$2:$H$26,E$1,$B$2:$B$26)</f>
+        <v/>
+      </c>
+      <c r="F30" s="16">
+        <f>SUMIF($H$2:$H$26,F$1,$B$2:$B$26)</f>
+        <v/>
+      </c>
+      <c r="G30" s="16">
+        <f>SUMIF($H$2:$H$26,G$1,$B$2:$B$26)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>這批貨的工時（分，1 site）</t>
+        </is>
+      </c>
+      <c r="C31" s="16">
+        <f>SUMPRODUCT((貨批!$B$2:$B$201=C$1)*貨批!$D$2:$D$201*貨批!$E$2:$E$201)/60</f>
+        <v/>
+      </c>
+      <c r="D31" s="16">
+        <f>SUMPRODUCT((貨批!$B$2:$B$201=D$1)*貨批!$D$2:$D$201*貨批!$E$2:$E$201)/60</f>
+        <v/>
+      </c>
+      <c r="E31" s="16">
+        <f>SUMPRODUCT((貨批!$B$2:$B$201=E$1)*貨批!$D$2:$D$201*貨批!$E$2:$E$201)/60</f>
+        <v/>
+      </c>
+      <c r="F31" s="16">
+        <f>SUMPRODUCT((貨批!$B$2:$B$201=F$1)*貨批!$D$2:$D$201*貨批!$E$2:$E$201)/60</f>
+        <v/>
+      </c>
+      <c r="G31" s="16">
+        <f>SUMPRODUCT((貨批!$B$2:$B$201=G$1)*貨批!$D$2:$D$201*貨批!$E$2:$E$201)/60</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="17" t="inlineStr">
+        <is>
+          <t>若完全不換 Kit，要跑幾小時</t>
+        </is>
+      </c>
+      <c r="C32" s="18">
+        <f>IFERROR(C31/C30/60,"—")</f>
+        <v/>
+      </c>
+      <c r="D32" s="18">
+        <f>IFERROR(D31/D30/60,"—")</f>
+        <v/>
+      </c>
+      <c r="E32" s="18">
+        <f>IFERROR(E31/E30/60,"—")</f>
+        <v/>
+      </c>
+      <c r="F32" s="18">
+        <f>IFERROR(F31/F30/60,"—")</f>
+        <v/>
+      </c>
+      <c r="G32" s="18">
+        <f>IFERROR(G31/G30/60,"—")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>✔ ＝ 這台機可以測這種封裝（對應「機台」分頁的 can_packages；空白代表該台什麼都能測，這裡會全部打勾）。</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>黃底 ＝ 這台機「現在」裝著的 Kit，也就是機隊此刻停在什麼配置。</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>最後一列是重點：把機隊凍結在現在的配置（完全不換 Kit），每種封裝各要跑多久。</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>哪一種明顯偏高，就是這批貨的瓶頸——代表它的量和現在裝著它的 site 數對不上，得先換 Kit 把配置拉回來。</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>這頁是對照用的，模擬器讀的仍然是「機台」分頁；改這裡不會改變模擬結果。</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Read machine capability from the matrix sheet when present
Ticking boxes beats editing "QFN48|QFN32" strings, so the 能力矩陣 sheet
now decides what each machine can run. The 機台 sheet still supplies the
machine list; drop the matrix sheet and capability falls back to
can_packages, as before.

Also fixes the sheet reader, which stacked rows in document order.
Excel omits fully blank rows, so a blank row vanished instead of leaving
a gap — and a blank row is exactly how the matrix separates its machine
rows from the summary and notes below. Rows now land at their real row
number, which also makes the row numbers in error messages correct.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TrwTqMZ3kHRLL23LGZ4TZk
</commit_message>
<xml_diff>
--- a/docs/模擬WIP_200批.xlsx
+++ b/docs/模擬WIP_200批.xlsx
@@ -10345,7 +10345,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J38"/>
+  <dimension ref="A1:J40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -11430,35 +11430,49 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>✔ ＝ 這台機可以測這種封裝（對應「機台」分頁的 can_packages；空白代表該台什麼都能測，這裡會全部打勾）。</t>
+          <t>✔ ＝ 這台機可以測這種封裝。要改就直接在格子裡打勾或清掉，模擬器以這頁為準。</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>黃底 ＝ 這台機「現在」裝著的 Kit，也就是機隊此刻停在什麼配置。</t>
+          <t>（打勾符號用 ✔ V O Y 1 都可以；留白或填 X 就是不能測。整列都沒勾＝視為全部都能測。）</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>最後一列是重點：把機隊凍結在現在的配置（完全不換 Kit），每種封裝各要跑多久。</t>
+          <t>黃底 ＝ 這台機「現在」裝著的 Kit，也就是機隊此刻停在什麼配置。</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>哪一種明顯偏高，就是這批貨的瓶頸——代表它的量和現在裝著它的 site 數對不上，得先換 Kit 把配置拉回來。</t>
+          <t>最後一列是重點：把機隊凍結在現在的配置（完全不換 Kit），每種封裝各要跑多久。</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>這頁是對照用的，模擬器讀的仍然是「機台」分頁；改這裡不會改變模擬結果。</t>
+          <t>哪一種明顯偏高，就是這批貨的瓶頸——代表它的量和現在裝著它的 site 數對不上，得先換 Kit 把配置拉回來。</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>刪掉整頁也可以，模擬器會改用「機台」分頁的 can_packages。</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>機台清單（台數、sites、目前 Kit、幾小時後可用）仍然以「機台」分頁為準，這頁只決定能力。</t>
         </is>
       </c>
     </row>

</xml_diff>